<commit_message>
Fix dynamic supporting healthcare headlines
</commit_message>
<xml_diff>
--- a/data/Resources and Terminology for Healthcare Indsutry Trends Website (6).xlsx
+++ b/data/Resources and Terminology for Healthcare Indsutry Trends Website (6).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/john_decicco_impact-advisors_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C161400-F001-46A4-8653-A4A07279B94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92D55196-0C72-4109-A36B-3D39D6D99A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{AE6C2486-B33D-41C7-9864-3BA3013F76A0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{AE6C2486-B33D-41C7-9864-3BA3013F76A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthcare Resources" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2431" uniqueCount="1228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2432" uniqueCount="1228">
   <si>
     <t xml:space="preserve">Title of Source </t>
   </si>
@@ -3289,6 +3289,9 @@
     <t>Supply chain reviews quarterly scorecards with a distributor to address low fill rates and recurring shipment errors.</t>
   </si>
   <si>
+    <t>Date Artcle Was Published</t>
+  </si>
+  <si>
     <t>The Role of Private Equity Funds in Healthcare: Trends, Impact, and Policy Responses</t>
   </si>
   <si>
@@ -3571,12 +3574,6 @@
     <t>Future success means treating revenue cycle as a strategic asset, not a support function | HFMA</t>
   </si>
   <si>
-    <t>Why AI Alone Fails in Healthcare and How AI+ Human Co-Management Drives Better Outcomes</t>
-  </si>
-  <si>
-    <t>Why AI Alone Fails in Healthcare and How AI + Human Co-Management Drives Better Outcomes | HFMA</t>
-  </si>
-  <si>
     <t>Medicare Claims Processing Modernization Gains Urgency At CMS</t>
   </si>
   <si>
@@ -3629,6 +3626,9 @@
   </si>
   <si>
     <t>AdaptHealth discloses patient data was stolen in cyberattack | Healthcare Dive</t>
+  </si>
+  <si>
+    <t>7/72026</t>
   </si>
   <si>
     <t>Private Equity May Skirt Oversight With Nonprofit Healthcare Joint Ventures</t>
@@ -3894,7 +3894,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3917,6 +3917,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4028,12 +4032,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E9F4E0EC-4852-4D2C-9BBE-852F6FF4678D}" name="Table1" displayName="Table1" ref="A1:C135" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="1" tableBorderDxfId="2">
-  <autoFilter ref="A1:C135" xr:uid="{E9F4E0EC-4852-4D2C-9BBE-852F6FF4678D}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E9F4E0EC-4852-4D2C-9BBE-852F6FF4678D}" name="Table1" displayName="Table1" ref="A1:D134" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:D134" xr:uid="{E9F4E0EC-4852-4D2C-9BBE-852F6FF4678D}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{6D3E6D37-6386-4019-A6CA-7BDAEBD1BE76}" name="Title of Source "/>
     <tableColumn id="2" xr3:uid="{86F8332B-8A32-497D-8E0C-91EF83BC9E63}" name="Website" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{5E9AB6AE-A04A-4E39-82CC-B13F8878BBCE}" name="Link to The Source " dataCellStyle="Hyperlink"/>
+    <tableColumn id="4" xr3:uid="{9F201A0B-5418-4CA9-8BB3-E1B8D6E9D937}" name="Date Artcle Was Published"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11386,15 +11391,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D0B573-CB40-455A-8450-09C524808966}">
-  <dimension ref="A1:C135"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="91.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="77.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.42578125" customWidth="1"/>
     <col min="3" max="3" width="155.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -11404,8 +11410,11 @@
       <c r="C1" s="17" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="16" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="7" t="s">
         <v>104</v>
       </c>
@@ -11415,8 +11424,11 @@
       <c r="C2" s="10" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2" s="18">
+        <v>45527</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
         <v>115</v>
       </c>
@@ -11426,8 +11438,11 @@
       <c r="C3" s="11" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3" s="18">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
         <v>117</v>
       </c>
@@ -11438,7 +11453,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
         <v>119</v>
       </c>
@@ -11448,8 +11463,11 @@
       <c r="C5" s="11" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5" s="18">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="7" t="s">
         <v>121</v>
       </c>
@@ -11459,8 +11477,11 @@
       <c r="C6" s="10" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6" s="18">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
         <v>123</v>
       </c>
@@ -11470,8 +11491,11 @@
       <c r="C7" s="11" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7" s="18">
+        <v>46076</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
         <v>125</v>
       </c>
@@ -11481,8 +11505,11 @@
       <c r="C8" s="10" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8" s="18">
+        <v>46049</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="9" t="s">
         <v>127</v>
       </c>
@@ -11492,8 +11519,11 @@
       <c r="C9" s="11" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9" s="18">
+        <v>45880</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="7" t="s">
         <v>129</v>
       </c>
@@ -11503,8 +11533,11 @@
       <c r="C10" s="10" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="D10" s="18">
+        <v>45511</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="9" t="s">
         <v>131</v>
       </c>
@@ -11514,8 +11547,11 @@
       <c r="C11" s="11" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="D11" s="18">
+        <v>45014</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="7" t="s">
         <v>133</v>
       </c>
@@ -11525,8 +11561,11 @@
       <c r="C12" s="10" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="D12" s="18">
+        <v>46007</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="9" t="s">
         <v>136</v>
       </c>
@@ -11536,8 +11575,11 @@
       <c r="C13" s="11" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="D13" s="18">
+        <v>45807</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="7" t="s">
         <v>141</v>
       </c>
@@ -11548,7 +11590,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:4">
       <c r="A15" s="9" t="s">
         <v>144</v>
       </c>
@@ -11559,7 +11601,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:4">
       <c r="A16" s="7" t="s">
         <v>146</v>
       </c>
@@ -11570,7 +11612,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:4">
       <c r="A17" s="9" t="s">
         <v>148</v>
       </c>
@@ -11580,8 +11622,11 @@
       <c r="C17" s="11" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
+      <c r="D17" s="18">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="7" t="s">
         <v>151</v>
       </c>
@@ -11591,8 +11636,11 @@
       <c r="C18" s="10" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="D18" s="18">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
         <v>154</v>
       </c>
@@ -11602,8 +11650,11 @@
       <c r="C19" s="11" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
+      <c r="D19" s="18">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="7" t="s">
         <v>156</v>
       </c>
@@ -11613,8 +11664,11 @@
       <c r="C20" s="10" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
+      <c r="D20" s="18">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
         <v>158</v>
       </c>
@@ -11624,8 +11678,11 @@
       <c r="C21" s="11" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="22" spans="1:3">
+      <c r="D21" s="18">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="7" t="s">
         <v>161</v>
       </c>
@@ -11635,8 +11692,11 @@
       <c r="C22" s="10" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="23" spans="1:3">
+      <c r="D22" s="18">
+        <v>45033</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
         <v>163</v>
       </c>
@@ -11646,8 +11706,11 @@
       <c r="C23" s="11" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="24" spans="1:3">
+      <c r="D23" s="18">
+        <v>45998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" s="7" t="s">
         <v>165</v>
       </c>
@@ -11657,8 +11720,11 @@
       <c r="C24" s="10" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="25" spans="1:3">
+      <c r="D24" s="18">
+        <v>45536</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="9" t="s">
         <v>167</v>
       </c>
@@ -11668,8 +11734,11 @@
       <c r="C25" s="11" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="26" spans="1:3">
+      <c r="D25" s="18">
+        <v>45742</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="7" t="s">
         <v>169</v>
       </c>
@@ -11679,8 +11748,11 @@
       <c r="C26" s="10" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="27" spans="1:3">
+      <c r="D26" s="18">
+        <v>45496</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="9" t="s">
         <v>171</v>
       </c>
@@ -11690,8 +11762,11 @@
       <c r="C27" s="11" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="28" spans="1:3">
+      <c r="D27" s="18">
+        <v>45089</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="7" t="s">
         <v>201</v>
       </c>
@@ -11701,8 +11776,11 @@
       <c r="C28" s="10" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="29" spans="1:3">
+      <c r="D28" s="18">
+        <v>45658</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
         <v>204</v>
       </c>
@@ -11712,8 +11790,11 @@
       <c r="C29" s="11" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
+      <c r="D29" s="18">
+        <v>45379</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="7" t="s">
         <v>206</v>
       </c>
@@ -11723,8 +11804,11 @@
       <c r="C30" s="10" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="31" spans="1:3">
+      <c r="D30" s="18">
+        <v>45512</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
         <v>208</v>
       </c>
@@ -11734,8 +11818,11 @@
       <c r="C31" s="11" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="32" spans="1:3">
+      <c r="D31">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="7" t="s">
         <v>211</v>
       </c>
@@ -11745,8 +11832,11 @@
       <c r="C32" s="10" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="33" spans="1:3">
+      <c r="D32" s="18">
+        <v>44046</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
         <v>214</v>
       </c>
@@ -11756,8 +11846,11 @@
       <c r="C33" s="11" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="D33" s="18">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34" s="7" t="s">
         <v>216</v>
       </c>
@@ -11767,8 +11860,11 @@
       <c r="C34" s="10" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="D34" s="18">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35" s="9" t="s">
         <v>218</v>
       </c>
@@ -11778,8 +11874,11 @@
       <c r="C35" s="11" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="36" spans="1:3">
+      <c r="D35" s="18">
+        <v>45435</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" s="7" t="s">
         <v>231</v>
       </c>
@@ -11790,7 +11889,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
         <v>233</v>
       </c>
@@ -11800,8 +11899,11 @@
       <c r="C37" s="11" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="38" spans="1:3">
+      <c r="D37" s="18">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" s="7" t="s">
         <v>235</v>
       </c>
@@ -11811,8 +11913,11 @@
       <c r="C38" s="10" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="39" spans="1:3">
+      <c r="D38" s="18">
+        <v>46085</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" s="9" t="s">
         <v>237</v>
       </c>
@@ -11822,8 +11927,11 @@
       <c r="C39" s="11" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="40" spans="1:3">
+      <c r="D39" s="18">
+        <v>46042</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40" s="7" t="s">
         <v>239</v>
       </c>
@@ -11833,8 +11941,11 @@
       <c r="C40" s="10" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="41" spans="1:3">
+      <c r="D40" s="18">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" s="9" t="s">
         <v>241</v>
       </c>
@@ -11844,8 +11955,11 @@
       <c r="C41" s="11" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="42" spans="1:3">
+      <c r="D41" s="18">
+        <v>45965</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" s="7" t="s">
         <v>252</v>
       </c>
@@ -11855,8 +11969,11 @@
       <c r="C42" s="10" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="43" spans="1:3">
+      <c r="D42" s="18">
+        <v>46091</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43" s="9" t="s">
         <v>255</v>
       </c>
@@ -11866,8 +11983,11 @@
       <c r="C43" s="11" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="44" spans="1:3">
+      <c r="D43" s="18">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" s="7" t="s">
         <v>257</v>
       </c>
@@ -11877,8 +11997,11 @@
       <c r="C44" s="10" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="45" spans="1:3">
+      <c r="D44" s="18">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" s="9" t="s">
         <v>259</v>
       </c>
@@ -11888,8 +12011,11 @@
       <c r="C45" s="11" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="46" spans="1:3">
+      <c r="D45" s="18">
+        <v>45391</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" s="7" t="s">
         <v>262</v>
       </c>
@@ -11899,8 +12025,11 @@
       <c r="C46" s="10" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="47" spans="1:3">
+      <c r="D46" s="18">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" s="9" t="s">
         <v>265</v>
       </c>
@@ -11910,8 +12039,11 @@
       <c r="C47" s="11" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="48" spans="1:3">
+      <c r="D47" s="18">
+        <v>45777</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" s="7" t="s">
         <v>267</v>
       </c>
@@ -11921,8 +12053,11 @@
       <c r="C48" s="10" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="49" spans="1:3">
+      <c r="D48" s="18">
+        <v>45239</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49" s="9" t="s">
         <v>270</v>
       </c>
@@ -11932,8 +12067,11 @@
       <c r="C49" s="11" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
+      <c r="D49" s="18">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" s="7" t="s">
         <v>290</v>
       </c>
@@ -11943,8 +12081,11 @@
       <c r="C50" s="10" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="51" spans="1:3">
+      <c r="D50" s="18">
+        <v>43319</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
       <c r="A51" s="9" t="s">
         <v>293</v>
       </c>
@@ -11954,8 +12095,11 @@
       <c r="C51" s="11" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="52" spans="1:3">
+      <c r="D51" s="18">
+        <v>43336</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
       <c r="A52" s="7" t="s">
         <v>295</v>
       </c>
@@ -11965,8 +12109,11 @@
       <c r="C52" s="10" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
+      <c r="D52" s="18">
+        <v>45707</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53" s="9" t="s">
         <v>298</v>
       </c>
@@ -11976,8 +12123,11 @@
       <c r="C53" s="11" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="54" spans="1:3">
+      <c r="D53" s="18">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54" s="7" t="s">
         <v>300</v>
       </c>
@@ -11987,8 +12137,11 @@
       <c r="C54" s="10" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="55" spans="1:3">
+      <c r="D54" s="18">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" s="9" t="s">
         <v>302</v>
       </c>
@@ -11999,7 +12152,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:4">
       <c r="A56" s="7" t="s">
         <v>305</v>
       </c>
@@ -12009,8 +12162,11 @@
       <c r="C56" s="10" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
+      <c r="D56" s="18">
+        <v>46187</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" s="9" t="s">
         <v>308</v>
       </c>
@@ -12020,8 +12176,11 @@
       <c r="C57" s="11" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="58" spans="1:3">
+      <c r="D57" s="18">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58" s="7" t="s">
         <v>311</v>
       </c>
@@ -12031,8 +12190,11 @@
       <c r="C58" s="10" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="59" spans="1:3">
+      <c r="D58" s="18">
+        <v>45685</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
       <c r="A59" s="9" t="s">
         <v>313</v>
       </c>
@@ -12043,7 +12205,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:4">
       <c r="A60" s="7" t="s">
         <v>315</v>
       </c>
@@ -12053,8 +12215,11 @@
       <c r="C60" s="10" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="61" spans="1:3">
+      <c r="D60" s="18">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
       <c r="A61" s="9" t="s">
         <v>318</v>
       </c>
@@ -12064,8 +12229,11 @@
       <c r="C61" s="11" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
+      <c r="D61" s="18">
+        <v>45870</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
       <c r="A62" s="7" t="s">
         <v>320</v>
       </c>
@@ -12075,8 +12243,11 @@
       <c r="C62" s="10" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="63" spans="1:3">
+      <c r="D62" s="18">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
       <c r="A63" s="9" t="s">
         <v>323</v>
       </c>
@@ -12086,8 +12257,11 @@
       <c r="C63" s="11" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="64" spans="1:3">
+      <c r="D63" s="18">
+        <v>45965</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
       <c r="A64" s="7" t="s">
         <v>325</v>
       </c>
@@ -12097,929 +12271,1127 @@
       <c r="C64" s="10" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="65" spans="1:3">
+      <c r="D64" s="18">
+        <v>44467</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
       <c r="A65" s="12" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B65" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>1084</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
+        <v>1085</v>
+      </c>
+      <c r="D65" s="18">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
       <c r="A66" s="14" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="B66" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>1086</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
+        <v>1087</v>
+      </c>
+      <c r="D66" s="18">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
       <c r="A67" s="3" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="B67" t="s">
         <v>105</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>1088</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
+        <v>1089</v>
+      </c>
+      <c r="D67" s="18">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
       <c r="A68" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="B68" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>1090</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3">
+        <v>1091</v>
+      </c>
+      <c r="D68" s="18">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B69" t="s">
         <v>105</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>1092</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3">
+        <v>1093</v>
+      </c>
+      <c r="D69" s="18">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="B70" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>1094</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3">
+        <v>1095</v>
+      </c>
+      <c r="D70" s="18">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="B71" t="s">
         <v>105</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>1096</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3">
+        <v>1097</v>
+      </c>
+      <c r="D71" s="18">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B72" s="13" t="s">
         <v>202</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>1098</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3">
+        <v>1099</v>
+      </c>
+      <c r="D72" s="18">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="B73" t="s">
         <v>202</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3">
+        <v>1101</v>
+      </c>
+      <c r="D73" s="18">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="B74" s="13" t="s">
         <v>202</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>1102</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
+        <v>1103</v>
+      </c>
+      <c r="D74" s="18">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="B75" t="s">
         <v>202</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>1104</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3">
+        <v>1105</v>
+      </c>
+      <c r="D75" s="18">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="B76" s="13" t="s">
         <v>202</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>1106</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3">
+        <v>1107</v>
+      </c>
+      <c r="D76" s="18">
+        <v>46180</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B77" t="s">
         <v>202</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>1108</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3">
+        <v>1109</v>
+      </c>
+      <c r="D77" s="18">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
       <c r="A78" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B78" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>1110</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3">
+        <v>1111</v>
+      </c>
+      <c r="D78" s="18">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
       <c r="A79" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="B79" t="s">
         <v>296</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>1112</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3">
+        <v>1113</v>
+      </c>
+      <c r="D79" s="18">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="B80" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>1114</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3">
+        <v>1115</v>
+      </c>
+      <c r="D80" s="18">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="B81" t="s">
         <v>296</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>1116</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3">
+        <v>1117</v>
+      </c>
+      <c r="D81" s="18">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B82" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>1118</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3">
+        <v>1119</v>
+      </c>
+      <c r="D82" s="18">
+        <v>45938</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="B83" t="s">
         <v>296</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>1120</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3">
+        <v>1121</v>
+      </c>
+      <c r="D83" s="18">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="B84" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>1122</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3">
+        <v>1123</v>
+      </c>
+      <c r="D84" s="18">
+        <v>46141</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
       <c r="A85" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="B85" t="s">
         <v>296</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>1124</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3">
+        <v>1125</v>
+      </c>
+      <c r="D85" s="18">
+        <v>46142</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="B86" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>1126</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3">
+        <v>1127</v>
+      </c>
+      <c r="D86" s="18">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B87" t="s">
         <v>296</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>1128</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3">
+        <v>1129</v>
+      </c>
+      <c r="D87" s="18">
+        <v>46129</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="B88" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>1130</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3">
+        <v>1131</v>
+      </c>
+      <c r="D88" s="18">
+        <v>46027</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
       <c r="A89" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="B89" t="s">
         <v>296</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>1132</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3">
+        <v>1133</v>
+      </c>
+      <c r="D89" s="18">
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
       <c r="A90" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="B90" s="13" t="s">
         <v>296</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>1134</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3">
+        <v>1135</v>
+      </c>
+      <c r="D90" s="18">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
       <c r="A91" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>149</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>1136</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3">
+        <v>1137</v>
+      </c>
+      <c r="D91" s="18">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="B92" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>1138</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3">
+        <v>1139</v>
+      </c>
+      <c r="D92" s="18">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
       <c r="A93" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B93" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>1140</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3">
+        <v>1141</v>
+      </c>
+      <c r="D93" s="18">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
       <c r="A94" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="B94" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>1142</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3">
+        <v>1143</v>
+      </c>
+      <c r="D94" s="18">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
       <c r="A95" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="B95" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>1144</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3">
+        <v>1145</v>
+      </c>
+      <c r="D95" s="18">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
       <c r="A96" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B96" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>1146</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3">
+        <v>1147</v>
+      </c>
+      <c r="D96" s="18">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
       <c r="A97" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="B97" s="13" t="s">
         <v>242</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>1148</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3">
+        <v>1149</v>
+      </c>
+      <c r="D97" s="18">
+        <v>46042</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
       <c r="A98" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="B98" t="s">
         <v>242</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>1150</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3">
+        <v>1151</v>
+      </c>
+      <c r="D98" s="18">
+        <v>46042</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="B99" s="13" t="s">
         <v>242</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>1152</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3">
+        <v>1153</v>
+      </c>
+      <c r="D99" s="18">
+        <v>46154</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
       <c r="A100" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B100" s="13" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>1155</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3">
+        <v>1156</v>
+      </c>
+      <c r="D100" s="18">
+        <v>45191</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
       <c r="A101" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="B101" s="13" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>1157</v>
       </c>
-      <c r="C101" s="1" t="s">
-        <v>1156</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3">
+    </row>
+    <row r="102" spans="1:4">
       <c r="A102" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>1160</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3">
+        <v>1161</v>
+      </c>
+      <c r="D102" s="18">
+        <v>45876</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="B103" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="104" spans="1:3">
+      <c r="D103" s="18">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4">
       <c r="A104" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="B104" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>1164</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3">
+        <v>1165</v>
+      </c>
+      <c r="D104" s="18">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4">
       <c r="A105" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>1166</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3">
+        <v>1167</v>
+      </c>
+      <c r="D105" s="18">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4">
       <c r="A106" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="B106" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>1168</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3">
+        <v>1169</v>
+      </c>
+      <c r="D106" s="18">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4">
       <c r="A107" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="B107" s="13" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3">
+        <v>1172</v>
+      </c>
+      <c r="D107" s="18">
+        <v>46075</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4">
       <c r="A108" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="B108" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>1173</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3">
+        <v>1174</v>
+      </c>
+      <c r="D108" s="18">
+        <v>46154</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4">
       <c r="A109" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="B109" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>1175</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3">
+        <v>1176</v>
+      </c>
+      <c r="D109" s="18">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4">
       <c r="A110" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B110" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>1177</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3">
+        <v>1178</v>
+      </c>
+      <c r="D110" s="18">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
       <c r="A111" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="B111" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>1179</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3">
+        <v>1180</v>
+      </c>
+      <c r="D111" s="18">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4">
       <c r="A112" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B112" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>1181</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3">
+        <v>1182</v>
+      </c>
+      <c r="D112" s="18">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
       <c r="A113" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="B113" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>1183</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3">
+        <v>1184</v>
+      </c>
+      <c r="D113" s="18">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
       <c r="A114" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="B114" s="13" t="s">
         <v>105</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>1185</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3">
+        <v>1186</v>
+      </c>
+      <c r="D114" s="18">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4">
       <c r="A115" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="B115" s="13" t="s">
-        <v>105</v>
+        <v>1163</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>1187</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3">
+        <v>1188</v>
+      </c>
+      <c r="D115" s="18">
+        <v>46231</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4">
       <c r="A116" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="B116" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>1189</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3">
+        <v>1190</v>
+      </c>
+      <c r="D116" s="18">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
       <c r="A117" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="B117" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>1191</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3">
+        <v>1192</v>
+      </c>
+      <c r="D117" s="18">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4">
       <c r="A118" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="B118" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>1193</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3">
+        <v>1194</v>
+      </c>
+      <c r="D118" s="19" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4">
       <c r="A119" t="s">
-        <v>1194</v>
+        <v>1196</v>
       </c>
       <c r="B119" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C119" s="1" t="s">
+        <v>1197</v>
+      </c>
+      <c r="D119" s="19" t="s">
         <v>1195</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:4">
       <c r="A120" t="s">
-        <v>1196</v>
+        <v>1198</v>
       </c>
       <c r="B120" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>1197</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3">
+        <v>1199</v>
+      </c>
+      <c r="D120" s="19" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4">
       <c r="A121" t="s">
-        <v>1198</v>
+        <v>1200</v>
       </c>
       <c r="B121" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>1199</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3">
+        <v>1201</v>
+      </c>
+      <c r="D121" s="18">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
       <c r="A122" t="s">
-        <v>1200</v>
+        <v>1202</v>
       </c>
       <c r="B122" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>1201</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3">
+        <v>1203</v>
+      </c>
+      <c r="D122" s="18">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4">
       <c r="A123" t="s">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="B123" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>1203</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3">
+        <v>1205</v>
+      </c>
+      <c r="D123" s="18">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
       <c r="A124" t="s">
-        <v>1204</v>
+        <v>1206</v>
       </c>
       <c r="B124" s="13" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>1205</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3">
+        <v>1207</v>
+      </c>
+      <c r="D124" s="18">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4">
       <c r="A125" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
       <c r="B125" s="13" t="s">
-        <v>1162</v>
+        <v>1209</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>1207</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3">
+        <v>1210</v>
+      </c>
+      <c r="D125" s="18">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4">
       <c r="A126" t="s">
-        <v>1208</v>
+        <v>1211</v>
       </c>
       <c r="B126" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>1210</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3">
+        <v>1212</v>
+      </c>
+      <c r="D126" s="18">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4">
       <c r="A127" t="s">
-        <v>1211</v>
+        <v>1213</v>
       </c>
       <c r="B127" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>1212</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3">
+        <v>349</v>
+      </c>
+      <c r="D127" s="18">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
       <c r="A128" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="B128" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3">
+        <v>1215</v>
+      </c>
+      <c r="D128" s="18">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
       <c r="A129" t="s">
-        <v>1214</v>
+        <v>1216</v>
       </c>
       <c r="B129" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>1215</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3">
+        <v>1217</v>
+      </c>
+      <c r="D129" s="18">
+        <v>46184</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4">
       <c r="A130" t="s">
-        <v>1216</v>
+        <v>1218</v>
       </c>
       <c r="B130" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>1217</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3">
+        <v>1219</v>
+      </c>
+      <c r="D130" s="18">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
       <c r="A131" t="s">
-        <v>1218</v>
+        <v>1220</v>
       </c>
       <c r="B131" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>1219</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3">
+        <v>1221</v>
+      </c>
+      <c r="D131" s="18">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
       <c r="A132" t="s">
-        <v>1220</v>
+        <v>1222</v>
       </c>
       <c r="B132" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>1221</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3">
+        <v>1223</v>
+      </c>
+      <c r="D132" s="18">
+        <v>46121</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
       <c r="A133" t="s">
-        <v>1222</v>
+        <v>1224</v>
       </c>
       <c r="B133" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>1223</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3">
+        <v>1225</v>
+      </c>
+      <c r="D133" s="18">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
       <c r="A134" t="s">
-        <v>1224</v>
+        <v>1226</v>
       </c>
       <c r="B134" s="13" t="s">
         <v>1209</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>1225</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" t="s">
-        <v>1226</v>
-      </c>
-      <c r="B135" s="13" t="s">
-        <v>1209</v>
-      </c>
-      <c r="C135" s="1" t="s">
         <v>1227</v>
+      </c>
+      <c r="D134" s="18">
+        <v>46071</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{B982DB95-FBE9-4EC0-922C-65C6E6EA9513}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{77FD4EF4-07FE-4261-9587-ADC58F010FF2}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{E1BAF727-8FE2-4017-BD4A-18813BC2FB6F}"/>
-    <hyperlink ref="C5" r:id="rId4" display="https://www.hfma.org/revenue-cycle/the-kpis-that-define-revenue-cycle-excellence/" xr:uid="{AFB97646-57E7-4F83-BC49-609EBA49CEA7}"/>
-    <hyperlink ref="C6" r:id="rId5" display="https://www.hfma.org/revenue-cycle/revenue-cycle-strategies-for-hospitals-facing-growing-financial-pressures/" xr:uid="{69CA50DC-862B-40E5-AFFC-43B29F592559}"/>
-    <hyperlink ref="C7" r:id="rId6" xr:uid="{99DF3E2A-53FD-4113-9FE7-CEAA852FB244}"/>
-    <hyperlink ref="C8" r:id="rId7" display="https://www.hfma.org/revenue-cycle/healthcare-providers-debate-ways-to-offer-patients-manageable-payment-options/" xr:uid="{18173A91-DAAE-4F7B-BA01-5E8E7D993389}"/>
-    <hyperlink ref="C9" r:id="rId8" display="https://www.hfma.org/reference/understand-claims-denial-friction/" xr:uid="{A1F1F68D-126E-4C00-9D46-AE3352C8D354}"/>
-    <hyperlink ref="C10" r:id="rId9" display="https://www.hfma.org/revenue-cycle/denials-management/navigating-the-rising-tide-of-denials/" xr:uid="{2CF6B11F-E233-458C-B70D-FC0F2121B5DC}"/>
-    <hyperlink ref="C11" r:id="rId10" display="https://www.hfma.org/revenue-cycle/denials-management/the-impact-of-claims-denials-on-the-financial-health-of-healthcare/" xr:uid="{AEC669AE-C71E-4C5A-8141-88040663F758}"/>
-    <hyperlink ref="C12" r:id="rId11" display="https://www.hfma.org/fast-finance/labor-outsourcing-shifts-to-non-clinical-roles/" xr:uid="{25B073F8-836E-4855-ADD8-A2A064BA7DE6}"/>
-    <hyperlink ref="C13" r:id="rId12" display="https://www.hfma.org/finance-and-business-strategy/why-labor-benchmarking-is-so-critical-to-healthcare-productivity/" xr:uid="{6ED3885E-89C5-4098-815B-89B7C9B25A3E}"/>
-    <hyperlink ref="C14" r:id="rId13" display="https://www.aha.org/guides-and-reports/2026-06-02-making-health-care-more-affordable" xr:uid="{90121FE9-87B7-4F7B-83C8-65DA125D03D4}"/>
-    <hyperlink ref="C15" r:id="rId14" display="https://www.aha.org/case-studies/2026-05-29-examples-how-hospitals-are-lowering-costs-and-enhancing-value" xr:uid="{FA927214-38B9-429E-A9B3-A8076BA89F07}"/>
-    <hyperlink ref="C16" r:id="rId15" display="https://www.aha.org/aha-center-health-innovation-market-scan/2026-01-05-/future-physician-workforce-optimization" xr:uid="{3A2526B7-D746-4D02-8BAA-80D9C22CBE09}"/>
-    <hyperlink ref="C17" r:id="rId16" display="https://www.beckershospitalreview.com/finance/revenue-cycle-management/5-recent-rcm-company-ma-moves/" xr:uid="{2336F0E4-D6BE-4B8F-80E4-CC4570DF336C}"/>
-    <hyperlink ref="C18" r:id="rId17" display="https://www.beckershospitalreview.com/finance/revenue-cycle-management/beyond-the-dashboard-why-the-most-damaging-denials-never-get-flagged/" xr:uid="{96B8AD2D-1B71-42FA-BB2B-0D4EE771A515}"/>
-    <hyperlink ref="C19" r:id="rId18" display="https://www.beckershospitalreview.com/healthcare-information-technology/ehrs/oracle-health-to-bring-ai-to-the-operating-room/" xr:uid="{8B730166-78F4-4E46-8A48-766E986D4590}"/>
-    <hyperlink ref="C20" r:id="rId19" display="https://www.beckershospitalreview.com/healthcare-information-technology/ehrs/will-ai-replace-physicians-epics-judy-faulkner-is-skeptical/" xr:uid="{0C1CEBEF-CE98-4DB5-B0C9-55AFF055DFFC}"/>
-    <hyperlink ref="C21" r:id="rId20" xr:uid="{E0C626A6-627F-4678-9B82-EA51DD8C470F}"/>
-    <hyperlink ref="C22" r:id="rId21" xr:uid="{C01CC20D-252E-4A9D-8A96-CC0A1D71C3B9}"/>
-    <hyperlink ref="C23" r:id="rId22" display="https://www.modernhealthcare.com/providers/mh-supply-chain-silos-amazon-business/" xr:uid="{EF2D6605-3F94-4E1D-B2A2-06F668E5301C}"/>
-    <hyperlink ref="C24" r:id="rId23" display="https://www.modernhealthcare.com/supply-chain/how-supply-chain-innovation-can-drive-efficiency-amid-cost-and-labor-headwinds/" xr:uid="{F1BCEC5C-260A-43D6-B7FB-C58A04305C1A}"/>
-    <hyperlink ref="C25" r:id="rId24" display="https://www.modernhealthcare.com/digital-health/ai-supply-chain-management-hospitals/" xr:uid="{5A3DB292-B129-4FA8-8FEC-FA8A425533AA}"/>
-    <hyperlink ref="C26" r:id="rId25" display="https://www.modernhealthcare.com/opinion/healthcare-consolidation-mergers-private-equity-james-calver/" xr:uid="{A80903FD-DA0C-45E7-88B8-DED70BBAF77A}"/>
-    <hyperlink ref="C27" r:id="rId26" display="https://www.modernhealthcare.com/safety-quality/how-hospitals-quality-improvements-shrinking-margins-leapfrog-group-CMS/" xr:uid="{8F5683F7-44A0-40A0-BDD5-819FA2CAEC17}"/>
-    <hyperlink ref="C28" r:id="rId27" display="https://www.mgma.com/articles/7-essential-components-of-a-high-performing-physician-enterprise" xr:uid="{15015813-0E75-4812-8F2E-55CEF2ABE697}"/>
-    <hyperlink ref="C29" r:id="rId28" display="https://www.mgma.com/articles/4-steps-for-creating-value-in-the-hospital-based-physician-enterprise" xr:uid="{7B3B65FA-DDC0-4EE1-A064-136509B7FD2C}"/>
-    <hyperlink ref="C30" r:id="rId29" display="https://www.mgma.com/articles/optimizing-physician-enterprise-performance-in-the-shift-to-value" xr:uid="{24034F1D-7957-422E-B20D-E246CDA1CD41}"/>
-    <hyperlink ref="C31" r:id="rId30" display="https://www.chartis.com/insights/why-time-has-come-evolve-physician-enterprise-roger-ray-md" xr:uid="{69FED3E0-0791-4AFF-BBA0-A2915D2509F3}"/>
-    <hyperlink ref="C32" r:id="rId31" display="https://nam.edu/perspectives/electronic-health-record-optimization-and-clinician-well-being-a-potential-roadmap-toward-action/" xr:uid="{07BADA26-2C9C-4CF2-BEB5-F009AF27CBA1}"/>
-    <hyperlink ref="C33" r:id="rId32" display="https://www.hfma.org/payment-reimbursement-and-managed-care/medicare-funding-projections-hi-trust-fund/" xr:uid="{726D89DF-6A5D-4470-9C86-DF2EEB69012B}"/>
-    <hyperlink ref="C34" r:id="rId33" display="https://www.hfma.org/payment-reimbursement-and-managed-care/medicare-payment-policy-changes-2027-hhs-hearings/" xr:uid="{B5D39D52-B9B5-4C31-8A2F-2765D05005B8}"/>
-    <hyperlink ref="C35" r:id="rId34" display="https://www.cdw.com/content/cdw/en/articles/digitalworkspace/how-clinical-workflow-optimization-creates-better-patient-outcomes.html?msockid=0a1b6b7b02a56ef323677c1e03966f9a" xr:uid="{66B75B10-FF64-419E-939B-C437F9A121CA}"/>
-    <hyperlink ref="C36" r:id="rId35" display="https://www.aha.org/aha-center-health-innovation-market-scan/2025-12-09-health-care-workforce-system-under-pressure-poised-reinvention" xr:uid="{4D560E3E-BD36-44CC-89D3-48378D5F72ED}"/>
-    <hyperlink ref="C37" r:id="rId36" display="https://www.modernhealthcare.com/politics-regulation/mh-us-health-spending-2034-cms/" xr:uid="{0CF95044-1CCF-4D79-90FC-C8274AC7A960}"/>
-    <hyperlink ref="C38" r:id="rId37" display="https://www.mgma.com/mgma-stat/keeping-your-clinician-productivity-on-track-throughout-2026" xr:uid="{38376598-160E-4122-9B39-6D6C0396A9D4}"/>
-    <hyperlink ref="C39" r:id="rId38" display="https://www.hfma.org/fast-finance/hospital-labor-trends-in-2025-show-slower-hiring-but-continued-workforce-growth/" xr:uid="{9878FDD7-6A47-467B-BA82-C735003F539D}"/>
-    <hyperlink ref="C40" r:id="rId39" display="https://www.hfma.org/how-a-health-system-can-reduce-premium-labor-while-building-a-sustainable-workforce/" xr:uid="{C4A314AA-0428-4FB4-905B-F638097E991C}"/>
-    <hyperlink ref="C41" r:id="rId40" display="https://www.ama-assn.org/practice-management/physician-health/when-health-care-teams-run-short-physician-burnout-rises" xr:uid="{4B625CF2-8597-46BB-998A-E06B2EB07402}"/>
-    <hyperlink ref="C42" r:id="rId41" xr:uid="{50837057-9C4C-459E-86AE-F8A65D62D99C}"/>
-    <hyperlink ref="C43" r:id="rId42" display="https://www.hfma.org/revenue-cycle/billing-and-collections/patient-pos-collections-pose-a-growing-rcm-problem/" xr:uid="{5438FC84-AD73-470B-AF61-E582BCAC9D80}"/>
-    <hyperlink ref="C44" r:id="rId43" display="https://www.hfma.org/revenue-cycle/billing-and-collections/prior-authorization-is-draining-revenue-which-is-why-automation-has-become-a-strategic-imperative/" xr:uid="{CF81E748-8C97-4D64-81B5-0844F2DD2D95}"/>
-    <hyperlink ref="C45" r:id="rId44" xr:uid="{060460A9-7A6E-4F65-ABDA-9E52B839A882}"/>
-    <hyperlink ref="C46" r:id="rId45" display="https://health.usnews.com/medicare/articles/your-guide-to-medicare-coverage" xr:uid="{49CFF0CC-F5ED-4038-AA6D-6C9436662F47}"/>
-    <hyperlink ref="C47" r:id="rId46" display="https://www.congress.gov/crs_external_products/R/PDF/R43357/R43357.21.pdf" xr:uid="{C69D2977-82CC-42D8-8196-CFA240CF9161}"/>
-    <hyperlink ref="C48" r:id="rId47" display="https://www.definitivehc.com/blog/the-difference-between-non-profit-and-for-profit-hospitals" xr:uid="{C4E6D896-AEA2-4156-9B19-157C6C82C422}"/>
-    <hyperlink ref="C49" r:id="rId48" display="https://www.healthcare-brew.com/stories/2025/09/29/difference-between-for-profit-nonprofit-hospitals" xr:uid="{318816D9-A902-4BA1-BF56-7B6F977CB130}"/>
-    <hyperlink ref="C50" r:id="rId49" display="https://www.ihi.org/library/blog/guiding-flock-3-simple-rules-improve-hospital-wide-patient-flow" xr:uid="{44313CC0-A1DA-471F-B790-A20B70405460}"/>
-    <hyperlink ref="C51" r:id="rId50" display="https://www.hfma.org/61738/" xr:uid="{BF46AE86-6158-44F6-B0E4-AA02A1FBB03E}"/>
-    <hyperlink ref="C52" r:id="rId51" display="https://www.kff.org/health-costs/key-facts-about-hospitals/" xr:uid="{CF8BD38B-1E9F-43EB-9F13-BAC58C834AC9}"/>
-    <hyperlink ref="C53" r:id="rId52" display="https://www.definitivehc.com/resources/healthcare-insights/hospital-operating-margins-united-states" xr:uid="{65B14E3D-ED45-4406-A012-E10D29E14174}"/>
-    <hyperlink ref="C54" r:id="rId53" display="https://www.beckershospitalreview.com/finance/from-2-2-to-16-5-36-health-systems-ranked-by-operating-margins-in-2025/" xr:uid="{23C82067-8E3E-4DB0-B203-096266095E3A}"/>
-    <hyperlink ref="C55" r:id="rId54" display="https://www.healthpartners.com/blog/medical-claim/" xr:uid="{3E3FEDC5-2489-438C-ACD2-D525FCD56387}"/>
-    <hyperlink ref="C56" r:id="rId55" display="https://www.medesk.net/en/blog/denial-management/" xr:uid="{592BF7EC-FFCA-4ACE-9148-DD9932CFC814}"/>
-    <hyperlink ref="C57" r:id="rId56" display="https://www.pgmbilling.com/blog/what-is-a-claim-scrubber-and-why-it-matters-more-than-ever/" xr:uid="{914634F4-692F-46C8-8291-E54A6E3331AF}"/>
-    <hyperlink ref="C58" r:id="rId57" display="https://healthcarereaders.com/insights/supply-chain-management-in-healthcare" xr:uid="{68BF8A32-144B-4916-949B-D71B4E67FD13}"/>
-    <hyperlink ref="C59" r:id="rId58" display="https://nihcm.org/publications/the-growth-of-private-equity-in-us-health-care-impact-and-outlook" xr:uid="{87FF73B9-EA0D-400F-A4FE-A372EF35BFDA}"/>
-    <hyperlink ref="C60" r:id="rId59" xr:uid="{E3A2D03F-A3B0-4419-BCC9-83B2A64BF450}"/>
-    <hyperlink ref="C61" r:id="rId60" display="https://www.definitivehc.com/resources/healthcare-insights/breaking-down-us-hospital-payor-mixes" xr:uid="{F056777D-BB12-462E-AFB4-35C81B489660}"/>
-    <hyperlink ref="C62" r:id="rId61" display="https://www.uhc.com/employer/news-strategies/annual-health-trends-report" xr:uid="{448F918A-0272-42AC-8111-FFC5E39012B6}"/>
-    <hyperlink ref="C63" r:id="rId62" display="https://publichealth.jhu.edu/2025/whats-behind-rising-health-insurance-costs" xr:uid="{FE9BDCF8-1682-401C-8799-60F27C681E8F}"/>
-    <hyperlink ref="C64" r:id="rId63" display="https://www.healthmarkets.com/resources/health-insurance/affordable-care-act-pros-and-cons" xr:uid="{3D578AA9-DE86-45F5-9003-740742DB790E}"/>
-    <hyperlink ref="C65" r:id="rId64" display="https://www.sciencedirect.com/science/article/pii/S0168851025001940" xr:uid="{70221E8B-AFC0-4159-94C9-2F06B0F95C1C}"/>
-    <hyperlink ref="C66" r:id="rId65" xr:uid="{78210D35-C927-4D02-93D0-1D002BB79C92}"/>
-    <hyperlink ref="C67" r:id="rId66" display="https://www.hfma.org/payment-reimbursement-and-managed-care/medicare-advantage-hospital-finances/" xr:uid="{06A39705-55DA-49F9-A4B1-A69081CD602C}"/>
-    <hyperlink ref="C68" r:id="rId67" display="https://www.hfma.org/accounting-and-financial-reporting/tax-exempt-hospital-reporting-requirements/" xr:uid="{5B236091-7DC0-4796-9E12-BA36C8B2FEEC}"/>
-    <hyperlink ref="C69" r:id="rId68" display="https://www.hfma.org/finance-and-business-strategy/hospital-drug-supply-costs/" xr:uid="{254AAC4F-0101-4F16-858B-203134B98D2C}"/>
-    <hyperlink ref="C70" r:id="rId69" display="https://www.hfma.org/payment-reimbursement-and-managed-care/contracting/white-house-zooms-in-on-hospital-contracts/" xr:uid="{4C7E1BC4-A0FB-42FC-A389-B3BC9FA33A5A}"/>
-    <hyperlink ref="C71" r:id="rId70" display="https://www.hfma.org/finance-and-business-strategy/healthcare-business-trends/the-hospital-of-the-future-with-jeni-williams/" xr:uid="{3559D1AC-00DD-4329-9C2F-AF32DB0C6A08}"/>
-    <hyperlink ref="C72" r:id="rId71" display="https://www.mgma.com/mgma-stat/stable-staff-to-physician-ratios-might-conceal-real-strain-in-your-practice" xr:uid="{FFE78512-8CFE-4DB0-A12B-63CC54B9F349}"/>
-    <hyperlink ref="C73" r:id="rId72" display="https://www.mgma.com/mgma-stat/revenue-growth-narrows-as-costs-climb-2026-squeeze" xr:uid="{740BC534-C9A0-4AF5-BB43-D0C526E6B8EF}"/>
-    <hyperlink ref="C74" r:id="rId73" display="https://www.mgma.com/mgma-stat/operating-costs-keep-climbing-for-medical-practices-in-2026" xr:uid="{7BE272E5-7AF4-4ECA-8513-C295270F72DD}"/>
-    <hyperlink ref="C75" r:id="rId74" display="https://www.mgma.com/mgma-stat/worker-benefits-where-retention-tools-meet-cost-pressure" xr:uid="{08F9AC08-815A-45A8-B58B-A3BDF2042DE6}"/>
-    <hyperlink ref="C76" r:id="rId75" display="https://www.mgma.com/articles/why-change-fails-in-medical-groups" xr:uid="{7D524D0A-460E-4DF2-97D7-BE22E57AD724}"/>
-    <hyperlink ref="C77" r:id="rId76" display="https://www.mgma.com/articles/designing-backfill-and-overbooking-by-specialty" xr:uid="{9B047851-BA08-4FE7-A9EC-40B367CE9084}"/>
-    <hyperlink ref="C78" r:id="rId77" display="https://www.kff.org/affordable-care-act/in-preliminary-rate-filings-aca-marketplace-insurers-largely-propose-double-digit-premium-increase-for-2027-following-a-steep-climb-this-year/" xr:uid="{95970B99-88DE-4B77-87D9-347DC113D924}"/>
-    <hyperlink ref="C79" r:id="rId78" display="https://www.kff.org/affordable-care-act/the-average-marketplace-deductible-grew-by-about-1000-per-person-in-2026-with-more-enrollees-shifting-to-higher-deductible-plans-as-enhanced-tax-credits-expired/" xr:uid="{F209C121-3B24-4230-B410-B0302E889464}"/>
-    <hyperlink ref="C80" r:id="rId79" display="https://www.kff.org/quick-insights/aca-marketplace-enrollment-is-down-by-3-million-after-big-jump-in-premium-payments/" xr:uid="{2AF6E803-CBA7-4B2B-9CB1-D02763DAAD8E}"/>
-    <hyperlink ref="C81" r:id="rId80" display="https://www.kff.org/health-costs/did-the-affordable-care-act-make-health-care-more-affordable/" xr:uid="{7BF8D13A-1412-481E-BF77-ECF0C5762002}"/>
-    <hyperlink ref="C82" r:id="rId81" display="https://www.kff.org/affordable-care-act/health-policy-101-the-affordable-care-act/" xr:uid="{8954F661-F310-4383-A271-A3B6083998C3}"/>
-    <hyperlink ref="C83" r:id="rId82" display="https://www.kff.org/health-costs/health-care-costs-keep-rising-why-and-who-pays/" xr:uid="{8AF914E6-E79E-49F5-8AFD-6F5BB9AAD1AF}"/>
-    <hyperlink ref="C84" r:id="rId83" display="https://www.kff.org/public-opinion/kff-health-tracking-poll-health-care-costs-and-the-midterms/" xr:uid="{1FBAD32A-EE4F-478A-9072-5F66C9110B7C}"/>
-    <hyperlink ref="C85" r:id="rId84" display="https://www.kff.org/health-costs/americans-challenges-with-health-care-costs/" xr:uid="{0835179D-699D-4646-9219-BCF3EE566F73}"/>
-    <hyperlink ref="C86" r:id="rId85" display="https://www.kff.org/health-costs/hospital-prices-have-risen-much-faster-for-private-insurance-than-medicare-since-2019/" xr:uid="{11B64026-B65B-4035-8D20-06B2616B3EA0}"/>
-    <hyperlink ref="C87" r:id="rId86" display="https://www.kff.org/health-costs/long-term-trends-in-employer-based-coverage/" xr:uid="{53DE45B8-B36B-48C1-8A56-2962301916DA}"/>
-    <hyperlink ref="C88" r:id="rId87" display="https://www.kff.org/patient-consumer-protections/policy-changes-bring-renewed-focus-on-high-deductible-health-plans/" xr:uid="{47351567-3580-473F-904C-B5A02F1B0E27}"/>
-    <hyperlink ref="C89" r:id="rId88" display="https://www.kff.org/health-costs/what-your-employer-based-health-coverage-really-costs/" xr:uid="{5492A1D3-EF9B-44EC-890B-BFD879A99B79}"/>
-    <hyperlink ref="C90" r:id="rId89" display="https://kffhealthnews.org/syndicate/long-term-care-costs-washington-state-payroll-option/" xr:uid="{E5E7EA74-3A13-45DC-807E-2C39C18FA09E}"/>
-    <hyperlink ref="B91" r:id="rId90" display="https://www.beckershospitalreview.com/finance/9-healthcare-bankruptcies-in-2026/" xr:uid="{4C7F5159-7C11-43CE-96A7-30E0E05D301B}"/>
-    <hyperlink ref="C91" r:id="rId91" display="https://www.beckershospitalreview.com/finance/9-healthcare-bankruptcies-in-2026/" xr:uid="{C0F1765B-90E7-4737-95E5-EDEAB043CB8A}"/>
-    <hyperlink ref="C92" r:id="rId92" display="https://www.beckershospitalreview.com/finance/hospital-margins-dip-to-2-9-average-as-expenses-grow-care-shifts-5-notes/" xr:uid="{2288C69D-2BC6-4042-88A1-1098651BE84E}"/>
-    <hyperlink ref="C93" r:id="rId93" display="https://www.beckershospitalreview.com/finance/the-term-payvider-makes-no-sense/" xr:uid="{BDB8C796-1019-4121-9F6C-F5AB08FA4A00}"/>
-    <hyperlink ref="C94" r:id="rId94" display="https://www.beckershospitalreview.com/finance/the-medicaid-squeeze-hospitals-cant-lobby-their-way-out-of/" xr:uid="{8C8318B2-32AD-4012-9AC0-FE729638B842}"/>
-    <hyperlink ref="C95" r:id="rId95" display="https://www.beckershospitalreview.com/healthcare-information-technology/ai/anthropics-claude-now-handles-healthcare-claims-care-management/" xr:uid="{CC7DEE30-3791-4535-86A1-2DCF199A6128}"/>
-    <hyperlink ref="C96" r:id="rId96" display="https://www.beckershospitalreview.com/healthcare-information-technology/ehrs/7-health-systems-moving-to-epic/" xr:uid="{3D8BDDF9-443A-44E7-93C2-42524C36BB97}"/>
-    <hyperlink ref="C97" r:id="rId97" display="https://edhub.ama-assn.org/steps-forward/audio-player/19032227?resultClick=1&amp;bypassSolrId=M_19032227" xr:uid="{4D8873B9-4680-4CF8-BF0E-E71871B1EABE}"/>
-    <hyperlink ref="C98" r:id="rId98" display="https://edhub.ama-assn.org/steps-forward/module/2844245?resultClick=1&amp;bypassSolrId=J_2844245" xr:uid="{96BA98DF-EC43-4DF1-B2FE-470B601ED37E}"/>
-    <hyperlink ref="C99" r:id="rId99" display="https://edhub.ama-assn.org/steps-forward/module/2781026?resultClick=1&amp;bypassSolrId=J_2781026" xr:uid="{F9943495-16D0-4890-920A-451B4BD5FB92}"/>
-    <hyperlink ref="C100" r:id="rId100" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10517477/" xr:uid="{B0184DD7-B152-4874-80EB-88A2AB606DD0}"/>
-    <hyperlink ref="C101" r:id="rId101" display="https://mayomagazine.mayoclinic.org/2026/04/ai-in-healthcare/" xr:uid="{C1240FFA-CAC6-49A2-BF9F-524C9F26FE7B}"/>
-    <hyperlink ref="C102" r:id="rId102" display="https://www.weforum.org/stories/health-and-healthcare-systems/ai-transforming-global-health/" xr:uid="{428F3DF0-A3A6-4C2F-B5B2-D88DB17F0A85}"/>
-    <hyperlink ref="C103" r:id="rId103" display="https://www.healthcaredive.com/spons/flipping-the-script-on-payer-denials-and-downcoding/824302/" xr:uid="{49F16536-227C-4254-A33E-E3622EEE0BC8}"/>
-    <hyperlink ref="C104" r:id="rId104" display="https://www.beckershospitalreview.com/finance/revenue-cycle-management/what-the-revenue-cycle-leaders-of-2030-will-know/" xr:uid="{53119244-DAA0-4B06-833B-1762966E5612}"/>
-    <hyperlink ref="C105" r:id="rId105" display="https://www.healthcaredive.com/spons/how-healthcare-ai-is-closing-the-revenue-gap/822195/" xr:uid="{03E774A3-278E-449A-8E64-7F75E033FC72}"/>
-    <hyperlink ref="C106" r:id="rId106" display="https://www.healthcaredive.com/news/himss-2026-takeaways-ai-innovation-agents-cybersecurity-governance-interoperability/814812/" xr:uid="{A34B8F48-E66E-4AC6-A388-558CA7A2D245}"/>
-    <hyperlink ref="C107" r:id="rId107" display="https://www.verywellhealth.com/health-insurance-for-multiple-states-4584359" xr:uid="{512E99DB-81FB-490E-A27C-B368DD14D8CC}"/>
-    <hyperlink ref="C108" r:id="rId108" display="https://www.hfma.org/technology/how-to-protect-revenue-in-a-digital-first-ecosystem/" xr:uid="{3A423EEB-CB75-485B-861F-8B93C1AD9DB1}"/>
-    <hyperlink ref="C109" r:id="rId109" display="https://www.hfma.org/technology/healthcare-revenue-cycle-transformation-three-priorities/" xr:uid="{30E0AFF3-5EA6-4CD1-94FB-905B6920D88B}"/>
-    <hyperlink ref="C110" r:id="rId110" display="https://www.hfma.org/technology/why-ai-alone-fails-in-healthcare-and-how-ai-human-co-management-drives-better-outcomes/" xr:uid="{DAE47884-B51E-4638-97B9-457EC83E1C8E}"/>
-    <hyperlink ref="C111" r:id="rId111" display="https://www.hfma.org/technology/medicare-claims-processing-modernization-cms/" xr:uid="{65E616D8-AEB8-435C-9AA4-22BB62F22DBC}"/>
-    <hyperlink ref="C112" r:id="rId112" display="https://www.hfma.org/revenue-cycle/modernize-your-operations-model-for-rcm-success/" xr:uid="{580A493E-9B72-438E-B317-4327030E645C}"/>
-    <hyperlink ref="C113" r:id="rId113" display="https://www.hfma.org/legal-and-regulatory-compliance/compliance/healthcare-fraud-compliance-cms-oversight/" xr:uid="{8A98ABB0-159B-4E33-A69F-A430692AAD6E}"/>
-    <hyperlink ref="C114" r:id="rId114" display="https://www.hfma.org/finance-and-business-strategy/building-a-more-effective-remittance-automation-strategy/" xr:uid="{970F056F-D30E-4B09-9450-32F576583FBC}"/>
-    <hyperlink ref="C115" r:id="rId115" display="https://www.hfma.org/finance-and-business-strategy/healthcare-affordability-financial-sustainability/" xr:uid="{554E107D-F704-49E5-BF8B-50FDB9FBEB3D}"/>
-    <hyperlink ref="C116" r:id="rId116" display="https://www.healthcaredive.com/news/tracking-healthcare-data-breaches-cybersecurity-hacking-hospitals/696184/" xr:uid="{5371A869-8E44-4A35-B84F-FABECC1C3C04}"/>
-    <hyperlink ref="C117" r:id="rId117" display="https://www.healthcaredive.com/news/affordable-care-act-premium-increase-2027-kff-peterson-center-healthcare/824695/" xr:uid="{B6F77715-FFAA-4275-B867-26D25D34D831}"/>
-    <hyperlink ref="C118" r:id="rId118" display="https://www.healthcaredive.com/news/epic-president-sumit-rana-step-down/824462/" xr:uid="{BA68F5CC-4C7D-4911-8AC0-EBC10B41F5DF}"/>
-    <hyperlink ref="C119" r:id="rId119" display="https://www.healthcaredive.com/news/adapthealth-discloses-patient-data-was-stolen-in-cyberattack/824601/" xr:uid="{7F1E13A2-B5AF-4522-89EA-756A9719C6EE}"/>
-    <hyperlink ref="C120" r:id="rId120" display="https://www.healthcaredive.com/news/private-equity-firms-may-skirt-healthcare-oversight-joint-ventures-nonprofits-pesp/824556/" xr:uid="{FA009102-A1D7-4124-828F-BD5E7558FB0C}"/>
-    <hyperlink ref="C121" r:id="rId121" display="https://www.healthcaredive.com/news/healthcare-faces-congressional-oversight-2026-midterms/824526/" xr:uid="{D90293DD-2974-4A65-A037-88E4FDC22785}"/>
-    <hyperlink ref="C122" r:id="rId122" display="https://www.healthcaredive.com/news/medicare-glp1-bridge-four-million-eligible-kff/824126/" xr:uid="{97E3F2B1-1C76-4584-BA72-374986F07B80}"/>
-    <hyperlink ref="C123" r:id="rId123" display="https://www.healthcaredive.com/news/us-health-spending-spikes-57t-2025/823660/" xr:uid="{F2000854-73E7-459F-9A02-7E24ADD05B01}"/>
-    <hyperlink ref="C124" r:id="rId124" display="https://www.healthcaredive.com/news/hackensack-meridian-hunterdon-explore-merger-nj-hospitals/823489/" xr:uid="{7C54EBAA-8A0E-4EC2-8235-6F2C0C3199EC}"/>
-    <hyperlink ref="C125" r:id="rId125" display="https://www.healthcaredive.com/news/centene-offers-employee-buyouts-membership-losses/823005/" xr:uid="{47565002-B618-4D8D-A378-2F0CF6B53B4F}"/>
-    <hyperlink ref="C126" r:id="rId126" display="https://www.healthaffairs.org/content/forefront/three-federal-streams-one-governance-problem-building-unified-ai-oversight-health" xr:uid="{EEFE2BB1-253E-4A5C-BA8E-49D7F45A6476}"/>
-    <hyperlink ref="C127" r:id="rId127" display="https://www.healthaffairs.org/content/forefront/medical-ethics-responds-private-equity" xr:uid="{981E0006-F1FB-4D04-8893-779D5F8F62B4}"/>
-    <hyperlink ref="C128" r:id="rId128" display="https://www.healthaffairs.org/doi/10.1377/hlthaff.2025.01325" xr:uid="{90091F37-B8BD-4BFC-A019-906839FABFB8}"/>
-    <hyperlink ref="C129" r:id="rId129" display="https://www.healthaffairs.org/content/forefront/states-exceeding-their-health-care-cost-growth-targets-does-mean" xr:uid="{07B09092-E3BB-4060-80CB-4D88E106A619}"/>
-    <hyperlink ref="C130" r:id="rId130" display="https://www.healthaffairs.org/content/forefront/why-new-drugs-and-ai-chatbots-won-t-cure-health-care-s-cost-disease" xr:uid="{4F073D69-1937-4F8D-8868-0CBA2A6219A7}"/>
-    <hyperlink ref="C131" r:id="rId131" display="https://www.healthaffairs.org/doi/10.1377/hlthaff.2026.00749" xr:uid="{3FAA25BD-2508-45E7-9827-E195A9CE2164}"/>
-    <hyperlink ref="C132" r:id="rId132" display="https://www.healthaffairs.org/content/forefront/cost-effectiveness-thresholds-overvaluing-innovation-undervaluing-health" xr:uid="{EC5E9BE7-5C6E-4049-A64D-C590235C2176}"/>
-    <hyperlink ref="C133" r:id="rId133" display="https://www.healthaffairs.org/content/forefront/levels-growth-and-semantics-role-prices-driving-health-care-spending" xr:uid="{1DD36C96-2124-485D-B38E-FD12539A44C2}"/>
-    <hyperlink ref="C134" r:id="rId134" display="https://www.healthaffairs.org/content/forefront/medicare-s-unrealized-opportunity-using-acos-create-real-competition" xr:uid="{A1AD029D-39C2-4AF6-8D1D-D213C93D7D93}"/>
-    <hyperlink ref="C135" r:id="rId135" display="https://www.healthaffairs.org/content/forefront/us-health-spending-problem-still-prices" xr:uid="{28D17A2C-13E5-42A2-BFB6-0A65FD4FFB24}"/>
+    <hyperlink ref="C5" r:id="rId3" display="https://www.hfma.org/revenue-cycle/the-kpis-that-define-revenue-cycle-excellence/" xr:uid="{AFB97646-57E7-4F83-BC49-609EBA49CEA7}"/>
+    <hyperlink ref="C6" r:id="rId4" display="https://www.hfma.org/revenue-cycle/revenue-cycle-strategies-for-hospitals-facing-growing-financial-pressures/" xr:uid="{69CA50DC-862B-40E5-AFFC-43B29F592559}"/>
+    <hyperlink ref="C7" r:id="rId5" xr:uid="{99DF3E2A-53FD-4113-9FE7-CEAA852FB244}"/>
+    <hyperlink ref="C8" r:id="rId6" display="https://www.hfma.org/revenue-cycle/healthcare-providers-debate-ways-to-offer-patients-manageable-payment-options/" xr:uid="{18173A91-DAAE-4F7B-BA01-5E8E7D993389}"/>
+    <hyperlink ref="C9" r:id="rId7" display="https://www.hfma.org/reference/understand-claims-denial-friction/" xr:uid="{A1F1F68D-126E-4C00-9D46-AE3352C8D354}"/>
+    <hyperlink ref="C10" r:id="rId8" display="https://www.hfma.org/revenue-cycle/denials-management/navigating-the-rising-tide-of-denials/" xr:uid="{2CF6B11F-E233-458C-B70D-FC0F2121B5DC}"/>
+    <hyperlink ref="C11" r:id="rId9" display="https://www.hfma.org/revenue-cycle/denials-management/the-impact-of-claims-denials-on-the-financial-health-of-healthcare/" xr:uid="{AEC669AE-C71E-4C5A-8141-88040663F758}"/>
+    <hyperlink ref="C12" r:id="rId10" display="https://www.hfma.org/fast-finance/labor-outsourcing-shifts-to-non-clinical-roles/" xr:uid="{25B073F8-836E-4855-ADD8-A2A064BA7DE6}"/>
+    <hyperlink ref="C13" r:id="rId11" display="https://www.hfma.org/finance-and-business-strategy/why-labor-benchmarking-is-so-critical-to-healthcare-productivity/" xr:uid="{6ED3885E-89C5-4098-815B-89B7C9B25A3E}"/>
+    <hyperlink ref="C14" r:id="rId12" display="https://www.aha.org/guides-and-reports/2026-06-02-making-health-care-more-affordable" xr:uid="{90121FE9-87B7-4F7B-83C8-65DA125D03D4}"/>
+    <hyperlink ref="C15" r:id="rId13" display="https://www.aha.org/case-studies/2026-05-29-examples-how-hospitals-are-lowering-costs-and-enhancing-value" xr:uid="{FA927214-38B9-429E-A9B3-A8076BA89F07}"/>
+    <hyperlink ref="C16" r:id="rId14" display="https://www.aha.org/aha-center-health-innovation-market-scan/2026-01-05-/future-physician-workforce-optimization" xr:uid="{3A2526B7-D746-4D02-8BAA-80D9C22CBE09}"/>
+    <hyperlink ref="C17" r:id="rId15" display="https://www.beckershospitalreview.com/finance/revenue-cycle-management/5-recent-rcm-company-ma-moves/" xr:uid="{2336F0E4-D6BE-4B8F-80E4-CC4570DF336C}"/>
+    <hyperlink ref="C18" r:id="rId16" display="https://www.beckershospitalreview.com/finance/revenue-cycle-management/beyond-the-dashboard-why-the-most-damaging-denials-never-get-flagged/" xr:uid="{96B8AD2D-1B71-42FA-BB2B-0D4EE771A515}"/>
+    <hyperlink ref="C19" r:id="rId17" display="https://www.beckershospitalreview.com/healthcare-information-technology/ehrs/oracle-health-to-bring-ai-to-the-operating-room/" xr:uid="{8B730166-78F4-4E46-8A48-766E986D4590}"/>
+    <hyperlink ref="C20" r:id="rId18" display="https://www.beckershospitalreview.com/healthcare-information-technology/ehrs/will-ai-replace-physicians-epics-judy-faulkner-is-skeptical/" xr:uid="{0C1CEBEF-CE98-4DB5-B0C9-55AFF055DFFC}"/>
+    <hyperlink ref="C21" r:id="rId19" xr:uid="{E0C626A6-627F-4678-9B82-EA51DD8C470F}"/>
+    <hyperlink ref="C22" r:id="rId20" xr:uid="{C01CC20D-252E-4A9D-8A96-CC0A1D71C3B9}"/>
+    <hyperlink ref="C23" r:id="rId21" display="https://www.modernhealthcare.com/providers/mh-supply-chain-silos-amazon-business/" xr:uid="{EF2D6605-3F94-4E1D-B2A2-06F668E5301C}"/>
+    <hyperlink ref="C24" r:id="rId22" display="https://www.modernhealthcare.com/supply-chain/how-supply-chain-innovation-can-drive-efficiency-amid-cost-and-labor-headwinds/" xr:uid="{F1BCEC5C-260A-43D6-B7FB-C58A04305C1A}"/>
+    <hyperlink ref="C25" r:id="rId23" display="https://www.modernhealthcare.com/digital-health/ai-supply-chain-management-hospitals/" xr:uid="{5A3DB292-B129-4FA8-8FEC-FA8A425533AA}"/>
+    <hyperlink ref="C26" r:id="rId24" display="https://www.modernhealthcare.com/opinion/healthcare-consolidation-mergers-private-equity-james-calver/" xr:uid="{A80903FD-DA0C-45E7-88B8-DED70BBAF77A}"/>
+    <hyperlink ref="C27" r:id="rId25" display="https://www.modernhealthcare.com/safety-quality/how-hospitals-quality-improvements-shrinking-margins-leapfrog-group-CMS/" xr:uid="{8F5683F7-44A0-40A0-BDD5-819FA2CAEC17}"/>
+    <hyperlink ref="C28" r:id="rId26" display="https://www.mgma.com/articles/7-essential-components-of-a-high-performing-physician-enterprise" xr:uid="{15015813-0E75-4812-8F2E-55CEF2ABE697}"/>
+    <hyperlink ref="C29" r:id="rId27" display="https://www.mgma.com/articles/4-steps-for-creating-value-in-the-hospital-based-physician-enterprise" xr:uid="{7B3B65FA-DDC0-4EE1-A064-136509B7FD2C}"/>
+    <hyperlink ref="C30" r:id="rId28" display="https://www.mgma.com/articles/optimizing-physician-enterprise-performance-in-the-shift-to-value" xr:uid="{24034F1D-7957-422E-B20D-E246CDA1CD41}"/>
+    <hyperlink ref="C31" r:id="rId29" display="https://www.chartis.com/insights/why-time-has-come-evolve-physician-enterprise-roger-ray-md" xr:uid="{69FED3E0-0791-4AFF-BBA0-A2915D2509F3}"/>
+    <hyperlink ref="C32" r:id="rId30" display="https://nam.edu/perspectives/electronic-health-record-optimization-and-clinician-well-being-a-potential-roadmap-toward-action/" xr:uid="{07BADA26-2C9C-4CF2-BEB5-F009AF27CBA1}"/>
+    <hyperlink ref="C33" r:id="rId31" display="https://www.hfma.org/payment-reimbursement-and-managed-care/medicare-funding-projections-hi-trust-fund/" xr:uid="{726D89DF-6A5D-4470-9C86-DF2EEB69012B}"/>
+    <hyperlink ref="C34" r:id="rId32" display="https://www.hfma.org/payment-reimbursement-and-managed-care/medicare-payment-policy-changes-2027-hhs-hearings/" xr:uid="{B5D39D52-B9B5-4C31-8A2F-2765D05005B8}"/>
+    <hyperlink ref="C35" r:id="rId33" display="https://www.cdw.com/content/cdw/en/articles/digitalworkspace/how-clinical-workflow-optimization-creates-better-patient-outcomes.html?msockid=0a1b6b7b02a56ef323677c1e03966f9a" xr:uid="{66B75B10-FF64-419E-939B-C437F9A121CA}"/>
+    <hyperlink ref="C36" r:id="rId34" display="https://www.aha.org/aha-center-health-innovation-market-scan/2025-12-09-health-care-workforce-system-under-pressure-poised-reinvention" xr:uid="{4D560E3E-BD36-44CC-89D3-48378D5F72ED}"/>
+    <hyperlink ref="C37" r:id="rId35" display="https://www.modernhealthcare.com/politics-regulation/mh-us-health-spending-2034-cms/" xr:uid="{0CF95044-1CCF-4D79-90FC-C8274AC7A960}"/>
+    <hyperlink ref="C38" r:id="rId36" display="https://www.mgma.com/mgma-stat/keeping-your-clinician-productivity-on-track-throughout-2026" xr:uid="{38376598-160E-4122-9B39-6D6C0396A9D4}"/>
+    <hyperlink ref="C39" r:id="rId37" display="https://www.hfma.org/fast-finance/hospital-labor-trends-in-2025-show-slower-hiring-but-continued-workforce-growth/" xr:uid="{9878FDD7-6A47-467B-BA82-C735003F539D}"/>
+    <hyperlink ref="C40" r:id="rId38" display="https://www.hfma.org/how-a-health-system-can-reduce-premium-labor-while-building-a-sustainable-workforce/" xr:uid="{C4A314AA-0428-4FB4-905B-F638097E991C}"/>
+    <hyperlink ref="C41" r:id="rId39" display="https://www.ama-assn.org/practice-management/physician-health/when-health-care-teams-run-short-physician-burnout-rises" xr:uid="{4B625CF2-8597-46BB-998A-E06B2EB07402}"/>
+    <hyperlink ref="C42" r:id="rId40" xr:uid="{50837057-9C4C-459E-86AE-F8A65D62D99C}"/>
+    <hyperlink ref="C43" r:id="rId41" display="https://www.hfma.org/revenue-cycle/billing-and-collections/patient-pos-collections-pose-a-growing-rcm-problem/" xr:uid="{5438FC84-AD73-470B-AF61-E582BCAC9D80}"/>
+    <hyperlink ref="C44" r:id="rId42" display="https://www.hfma.org/revenue-cycle/billing-and-collections/prior-authorization-is-draining-revenue-which-is-why-automation-has-become-a-strategic-imperative/" xr:uid="{CF81E748-8C97-4D64-81B5-0844F2DD2D95}"/>
+    <hyperlink ref="C45" r:id="rId43" xr:uid="{060460A9-7A6E-4F65-ABDA-9E52B839A882}"/>
+    <hyperlink ref="C46" r:id="rId44" display="https://health.usnews.com/medicare/articles/your-guide-to-medicare-coverage" xr:uid="{49CFF0CC-F5ED-4038-AA6D-6C9436662F47}"/>
+    <hyperlink ref="C47" r:id="rId45" display="https://www.congress.gov/crs_external_products/R/PDF/R43357/R43357.21.pdf" xr:uid="{C69D2977-82CC-42D8-8196-CFA240CF9161}"/>
+    <hyperlink ref="C48" r:id="rId46" display="https://www.definitivehc.com/blog/the-difference-between-non-profit-and-for-profit-hospitals" xr:uid="{C4E6D896-AEA2-4156-9B19-157C6C82C422}"/>
+    <hyperlink ref="C49" r:id="rId47" display="https://www.healthcare-brew.com/stories/2025/09/29/difference-between-for-profit-nonprofit-hospitals" xr:uid="{318816D9-A902-4BA1-BF56-7B6F977CB130}"/>
+    <hyperlink ref="C50" r:id="rId48" display="https://www.ihi.org/library/blog/guiding-flock-3-simple-rules-improve-hospital-wide-patient-flow" xr:uid="{44313CC0-A1DA-471F-B790-A20B70405460}"/>
+    <hyperlink ref="C51" r:id="rId49" display="https://www.hfma.org/61738/" xr:uid="{BF46AE86-6158-44F6-B0E4-AA02A1FBB03E}"/>
+    <hyperlink ref="C52" r:id="rId50" display="https://www.kff.org/health-costs/key-facts-about-hospitals/" xr:uid="{CF8BD38B-1E9F-43EB-9F13-BAC58C834AC9}"/>
+    <hyperlink ref="C53" r:id="rId51" display="https://www.definitivehc.com/resources/healthcare-insights/hospital-operating-margins-united-states" xr:uid="{65B14E3D-ED45-4406-A012-E10D29E14174}"/>
+    <hyperlink ref="C54" r:id="rId52" display="https://www.beckershospitalreview.com/finance/from-2-2-to-16-5-36-health-systems-ranked-by-operating-margins-in-2025/" xr:uid="{23C82067-8E3E-4DB0-B203-096266095E3A}"/>
+    <hyperlink ref="C55" r:id="rId53" display="https://www.healthpartners.com/blog/medical-claim/" xr:uid="{3E3FEDC5-2489-438C-ACD2-D525FCD56387}"/>
+    <hyperlink ref="C56" r:id="rId54" display="https://www.medesk.net/en/blog/denial-management/" xr:uid="{592BF7EC-FFCA-4ACE-9148-DD9932CFC814}"/>
+    <hyperlink ref="C57" r:id="rId55" display="https://www.pgmbilling.com/blog/what-is-a-claim-scrubber-and-why-it-matters-more-than-ever/" xr:uid="{914634F4-692F-46C8-8291-E54A6E3331AF}"/>
+    <hyperlink ref="C58" r:id="rId56" display="https://healthcarereaders.com/insights/supply-chain-management-in-healthcare" xr:uid="{68BF8A32-144B-4916-949B-D71B4E67FD13}"/>
+    <hyperlink ref="C59" r:id="rId57" display="https://nihcm.org/publications/the-growth-of-private-equity-in-us-health-care-impact-and-outlook" xr:uid="{87FF73B9-EA0D-400F-A4FE-A372EF35BFDA}"/>
+    <hyperlink ref="C60" r:id="rId58" xr:uid="{E3A2D03F-A3B0-4419-BCC9-83B2A64BF450}"/>
+    <hyperlink ref="C61" r:id="rId59" display="https://www.definitivehc.com/resources/healthcare-insights/breaking-down-us-hospital-payor-mixes" xr:uid="{F056777D-BB12-462E-AFB4-35C81B489660}"/>
+    <hyperlink ref="C62" r:id="rId60" display="https://www.uhc.com/employer/news-strategies/annual-health-trends-report" xr:uid="{448F918A-0272-42AC-8111-FFC5E39012B6}"/>
+    <hyperlink ref="C63" r:id="rId61" display="https://publichealth.jhu.edu/2025/whats-behind-rising-health-insurance-costs" xr:uid="{FE9BDCF8-1682-401C-8799-60F27C681E8F}"/>
+    <hyperlink ref="C64" r:id="rId62" display="https://www.healthmarkets.com/resources/health-insurance/affordable-care-act-pros-and-cons" xr:uid="{3D578AA9-DE86-45F5-9003-740742DB790E}"/>
+    <hyperlink ref="C65" r:id="rId63" display="https://www.sciencedirect.com/science/article/pii/S0168851025001940" xr:uid="{70221E8B-AFC0-4159-94C9-2F06B0F95C1C}"/>
+    <hyperlink ref="C66" r:id="rId64" xr:uid="{78210D35-C927-4D02-93D0-1D002BB79C92}"/>
+    <hyperlink ref="C67" r:id="rId65" display="https://www.hfma.org/payment-reimbursement-and-managed-care/medicare-advantage-hospital-finances/" xr:uid="{06A39705-55DA-49F9-A4B1-A69081CD602C}"/>
+    <hyperlink ref="C68" r:id="rId66" display="https://www.hfma.org/accounting-and-financial-reporting/tax-exempt-hospital-reporting-requirements/" xr:uid="{5B236091-7DC0-4796-9E12-BA36C8B2FEEC}"/>
+    <hyperlink ref="C69" r:id="rId67" display="https://www.hfma.org/finance-and-business-strategy/hospital-drug-supply-costs/" xr:uid="{254AAC4F-0101-4F16-858B-203134B98D2C}"/>
+    <hyperlink ref="C70" r:id="rId68" display="https://www.hfma.org/payment-reimbursement-and-managed-care/contracting/white-house-zooms-in-on-hospital-contracts/" xr:uid="{4C7E1BC4-A0FB-42FC-A389-B3BC9FA33A5A}"/>
+    <hyperlink ref="C71" r:id="rId69" display="https://www.hfma.org/finance-and-business-strategy/healthcare-business-trends/the-hospital-of-the-future-with-jeni-williams/" xr:uid="{3559D1AC-00DD-4329-9C2F-AF32DB0C6A08}"/>
+    <hyperlink ref="C72" r:id="rId70" display="https://www.mgma.com/mgma-stat/stable-staff-to-physician-ratios-might-conceal-real-strain-in-your-practice" xr:uid="{FFE78512-8CFE-4DB0-A12B-63CC54B9F349}"/>
+    <hyperlink ref="C73" r:id="rId71" display="https://www.mgma.com/mgma-stat/revenue-growth-narrows-as-costs-climb-2026-squeeze" xr:uid="{740BC534-C9A0-4AF5-BB43-D0C526E6B8EF}"/>
+    <hyperlink ref="C74" r:id="rId72" display="https://www.mgma.com/mgma-stat/operating-costs-keep-climbing-for-medical-practices-in-2026" xr:uid="{7BE272E5-7AF4-4ECA-8513-C295270F72DD}"/>
+    <hyperlink ref="C75" r:id="rId73" display="https://www.mgma.com/mgma-stat/worker-benefits-where-retention-tools-meet-cost-pressure" xr:uid="{08F9AC08-815A-45A8-B58B-A3BDF2042DE6}"/>
+    <hyperlink ref="C76" r:id="rId74" display="https://www.mgma.com/articles/why-change-fails-in-medical-groups" xr:uid="{7D524D0A-460E-4DF2-97D7-BE22E57AD724}"/>
+    <hyperlink ref="C77" r:id="rId75" display="https://www.mgma.com/articles/designing-backfill-and-overbooking-by-specialty" xr:uid="{9B047851-BA08-4FE7-A9EC-40B367CE9084}"/>
+    <hyperlink ref="C78" r:id="rId76" display="https://www.kff.org/affordable-care-act/in-preliminary-rate-filings-aca-marketplace-insurers-largely-propose-double-digit-premium-increase-for-2027-following-a-steep-climb-this-year/" xr:uid="{95970B99-88DE-4B77-87D9-347DC113D924}"/>
+    <hyperlink ref="C79" r:id="rId77" display="https://www.kff.org/affordable-care-act/the-average-marketplace-deductible-grew-by-about-1000-per-person-in-2026-with-more-enrollees-shifting-to-higher-deductible-plans-as-enhanced-tax-credits-expired/" xr:uid="{F209C121-3B24-4230-B410-B0302E889464}"/>
+    <hyperlink ref="C80" r:id="rId78" display="https://www.kff.org/quick-insights/aca-marketplace-enrollment-is-down-by-3-million-after-big-jump-in-premium-payments/" xr:uid="{2AF6E803-CBA7-4B2B-9CB1-D02763DAAD8E}"/>
+    <hyperlink ref="C81" r:id="rId79" display="https://www.kff.org/health-costs/did-the-affordable-care-act-make-health-care-more-affordable/" xr:uid="{7BF8D13A-1412-481E-BF77-ECF0C5762002}"/>
+    <hyperlink ref="C82" r:id="rId80" display="https://www.kff.org/affordable-care-act/health-policy-101-the-affordable-care-act/" xr:uid="{8954F661-F310-4383-A271-A3B6083998C3}"/>
+    <hyperlink ref="C83" r:id="rId81" display="https://www.kff.org/health-costs/health-care-costs-keep-rising-why-and-who-pays/" xr:uid="{8AF914E6-E79E-49F5-8AFD-6F5BB9AAD1AF}"/>
+    <hyperlink ref="C84" r:id="rId82" display="https://www.kff.org/public-opinion/kff-health-tracking-poll-health-care-costs-and-the-midterms/" xr:uid="{1FBAD32A-EE4F-478A-9072-5F66C9110B7C}"/>
+    <hyperlink ref="C85" r:id="rId83" display="https://www.kff.org/health-costs/americans-challenges-with-health-care-costs/" xr:uid="{0835179D-699D-4646-9219-BCF3EE566F73}"/>
+    <hyperlink ref="C86" r:id="rId84" display="https://www.kff.org/health-costs/hospital-prices-have-risen-much-faster-for-private-insurance-than-medicare-since-2019/" xr:uid="{11B64026-B65B-4035-8D20-06B2616B3EA0}"/>
+    <hyperlink ref="C87" r:id="rId85" display="https://www.kff.org/health-costs/long-term-trends-in-employer-based-coverage/" xr:uid="{53DE45B8-B36B-48C1-8A56-2962301916DA}"/>
+    <hyperlink ref="C88" r:id="rId86" display="https://www.kff.org/patient-consumer-protections/policy-changes-bring-renewed-focus-on-high-deductible-health-plans/" xr:uid="{47351567-3580-473F-904C-B5A02F1B0E27}"/>
+    <hyperlink ref="C89" r:id="rId87" display="https://www.kff.org/health-costs/what-your-employer-based-health-coverage-really-costs/" xr:uid="{5492A1D3-EF9B-44EC-890B-BFD879A99B79}"/>
+    <hyperlink ref="C90" r:id="rId88" display="https://kffhealthnews.org/syndicate/long-term-care-costs-washington-state-payroll-option/" xr:uid="{E5E7EA74-3A13-45DC-807E-2C39C18FA09E}"/>
+    <hyperlink ref="B91" r:id="rId89" display="https://www.beckershospitalreview.com/finance/9-healthcare-bankruptcies-in-2026/" xr:uid="{4C7F5159-7C11-43CE-96A7-30E0E05D301B}"/>
+    <hyperlink ref="C91" r:id="rId90" display="https://www.beckershospitalreview.com/finance/9-healthcare-bankruptcies-in-2026/" xr:uid="{C0F1765B-90E7-4737-95E5-EDEAB043CB8A}"/>
+    <hyperlink ref="C92" r:id="rId91" display="https://www.beckershospitalreview.com/finance/hospital-margins-dip-to-2-9-average-as-expenses-grow-care-shifts-5-notes/" xr:uid="{2288C69D-2BC6-4042-88A1-1098651BE84E}"/>
+    <hyperlink ref="C93" r:id="rId92" display="https://www.beckershospitalreview.com/finance/the-term-payvider-makes-no-sense/" xr:uid="{BDB8C796-1019-4121-9F6C-F5AB08FA4A00}"/>
+    <hyperlink ref="C94" r:id="rId93" display="https://www.beckershospitalreview.com/finance/the-medicaid-squeeze-hospitals-cant-lobby-their-way-out-of/" xr:uid="{8C8318B2-32AD-4012-9AC0-FE729638B842}"/>
+    <hyperlink ref="C95" r:id="rId94" display="https://www.beckershospitalreview.com/healthcare-information-technology/ai/anthropics-claude-now-handles-healthcare-claims-care-management/" xr:uid="{CC7DEE30-3791-4535-86A1-2DCF199A6128}"/>
+    <hyperlink ref="C96" r:id="rId95" display="https://www.beckershospitalreview.com/healthcare-information-technology/ehrs/7-health-systems-moving-to-epic/" xr:uid="{3D8BDDF9-443A-44E7-93C2-42524C36BB97}"/>
+    <hyperlink ref="C97" r:id="rId96" display="https://edhub.ama-assn.org/steps-forward/audio-player/19032227?resultClick=1&amp;bypassSolrId=M_19032227" xr:uid="{4D8873B9-4680-4CF8-BF0E-E71871B1EABE}"/>
+    <hyperlink ref="C98" r:id="rId97" display="https://edhub.ama-assn.org/steps-forward/module/2844245?resultClick=1&amp;bypassSolrId=J_2844245" xr:uid="{96BA98DF-EC43-4DF1-B2FE-470B601ED37E}"/>
+    <hyperlink ref="C99" r:id="rId98" display="https://edhub.ama-assn.org/steps-forward/module/2781026?resultClick=1&amp;bypassSolrId=J_2781026" xr:uid="{F9943495-16D0-4890-920A-451B4BD5FB92}"/>
+    <hyperlink ref="C100" r:id="rId99" display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10517477/" xr:uid="{B0184DD7-B152-4874-80EB-88A2AB606DD0}"/>
+    <hyperlink ref="C101" r:id="rId100" display="https://mayomagazine.mayoclinic.org/2026/04/ai-in-healthcare/" xr:uid="{C1240FFA-CAC6-49A2-BF9F-524C9F26FE7B}"/>
+    <hyperlink ref="C102" r:id="rId101" display="https://www.weforum.org/stories/health-and-healthcare-systems/ai-transforming-global-health/" xr:uid="{428F3DF0-A3A6-4C2F-B5B2-D88DB17F0A85}"/>
+    <hyperlink ref="C103" r:id="rId102" display="https://www.healthcaredive.com/spons/flipping-the-script-on-payer-denials-and-downcoding/824302/" xr:uid="{49F16536-227C-4254-A33E-E3622EEE0BC8}"/>
+    <hyperlink ref="C104" r:id="rId103" display="https://www.beckershospitalreview.com/finance/revenue-cycle-management/what-the-revenue-cycle-leaders-of-2030-will-know/" xr:uid="{53119244-DAA0-4B06-833B-1762966E5612}"/>
+    <hyperlink ref="C105" r:id="rId104" display="https://www.healthcaredive.com/spons/how-healthcare-ai-is-closing-the-revenue-gap/822195/" xr:uid="{03E774A3-278E-449A-8E64-7F75E033FC72}"/>
+    <hyperlink ref="C106" r:id="rId105" display="https://www.healthcaredive.com/news/himss-2026-takeaways-ai-innovation-agents-cybersecurity-governance-interoperability/814812/" xr:uid="{A34B8F48-E66E-4AC6-A388-558CA7A2D245}"/>
+    <hyperlink ref="C107" r:id="rId106" display="https://www.verywellhealth.com/health-insurance-for-multiple-states-4584359" xr:uid="{512E99DB-81FB-490E-A27C-B368DD14D8CC}"/>
+    <hyperlink ref="C108" r:id="rId107" display="https://www.hfma.org/technology/how-to-protect-revenue-in-a-digital-first-ecosystem/" xr:uid="{3A423EEB-CB75-485B-861F-8B93C1AD9DB1}"/>
+    <hyperlink ref="C109" r:id="rId108" display="https://www.hfma.org/technology/healthcare-revenue-cycle-transformation-three-priorities/" xr:uid="{30E0AFF3-5EA6-4CD1-94FB-905B6920D88B}"/>
+    <hyperlink ref="C110" r:id="rId109" display="https://www.hfma.org/technology/medicare-claims-processing-modernization-cms/" xr:uid="{65E616D8-AEB8-435C-9AA4-22BB62F22DBC}"/>
+    <hyperlink ref="C111" r:id="rId110" display="https://www.hfma.org/revenue-cycle/modernize-your-operations-model-for-rcm-success/" xr:uid="{580A493E-9B72-438E-B317-4327030E645C}"/>
+    <hyperlink ref="C112" r:id="rId111" display="https://www.hfma.org/legal-and-regulatory-compliance/compliance/healthcare-fraud-compliance-cms-oversight/" xr:uid="{8A98ABB0-159B-4E33-A69F-A430692AAD6E}"/>
+    <hyperlink ref="C113" r:id="rId112" display="https://www.hfma.org/finance-and-business-strategy/building-a-more-effective-remittance-automation-strategy/" xr:uid="{970F056F-D30E-4B09-9450-32F576583FBC}"/>
+    <hyperlink ref="C114" r:id="rId113" display="https://www.hfma.org/finance-and-business-strategy/healthcare-affordability-financial-sustainability/" xr:uid="{554E107D-F704-49E5-BF8B-50FDB9FBEB3D}"/>
+    <hyperlink ref="C115" r:id="rId114" display="https://www.healthcaredive.com/news/tracking-healthcare-data-breaches-cybersecurity-hacking-hospitals/696184/" xr:uid="{5371A869-8E44-4A35-B84F-FABECC1C3C04}"/>
+    <hyperlink ref="C116" r:id="rId115" display="https://www.healthcaredive.com/news/affordable-care-act-premium-increase-2027-kff-peterson-center-healthcare/824695/" xr:uid="{B6F77715-FFAA-4275-B867-26D25D34D831}"/>
+    <hyperlink ref="C117" r:id="rId116" display="https://www.healthcaredive.com/news/epic-president-sumit-rana-step-down/824462/" xr:uid="{BA68F5CC-4C7D-4911-8AC0-EBC10B41F5DF}"/>
+    <hyperlink ref="C118" r:id="rId117" display="https://www.healthcaredive.com/news/adapthealth-discloses-patient-data-was-stolen-in-cyberattack/824601/" xr:uid="{7F1E13A2-B5AF-4522-89EA-756A9719C6EE}"/>
+    <hyperlink ref="C119" r:id="rId118" display="https://www.healthcaredive.com/news/private-equity-firms-may-skirt-healthcare-oversight-joint-ventures-nonprofits-pesp/824556/" xr:uid="{FA009102-A1D7-4124-828F-BD5E7558FB0C}"/>
+    <hyperlink ref="C120" r:id="rId119" display="https://www.healthcaredive.com/news/healthcare-faces-congressional-oversight-2026-midterms/824526/" xr:uid="{D90293DD-2974-4A65-A037-88E4FDC22785}"/>
+    <hyperlink ref="C121" r:id="rId120" display="https://www.healthcaredive.com/news/medicare-glp1-bridge-four-million-eligible-kff/824126/" xr:uid="{97E3F2B1-1C76-4584-BA72-374986F07B80}"/>
+    <hyperlink ref="C122" r:id="rId121" display="https://www.healthcaredive.com/news/us-health-spending-spikes-57t-2025/823660/" xr:uid="{F2000854-73E7-459F-9A02-7E24ADD05B01}"/>
+    <hyperlink ref="C123" r:id="rId122" display="https://www.healthcaredive.com/news/hackensack-meridian-hunterdon-explore-merger-nj-hospitals/823489/" xr:uid="{7C54EBAA-8A0E-4EC2-8235-6F2C0C3199EC}"/>
+    <hyperlink ref="C124" r:id="rId123" display="https://www.healthcaredive.com/news/centene-offers-employee-buyouts-membership-losses/823005/" xr:uid="{47565002-B618-4D8D-A378-2F0CF6B53B4F}"/>
+    <hyperlink ref="C125" r:id="rId124" display="https://www.healthaffairs.org/content/forefront/three-federal-streams-one-governance-problem-building-unified-ai-oversight-health" xr:uid="{EEFE2BB1-253E-4A5C-BA8E-49D7F45A6476}"/>
+    <hyperlink ref="C126" r:id="rId125" display="https://www.healthaffairs.org/content/forefront/medical-ethics-responds-private-equity" xr:uid="{981E0006-F1FB-4D04-8893-779D5F8F62B4}"/>
+    <hyperlink ref="C127" r:id="rId126" display="https://www.healthaffairs.org/doi/10.1377/hlthaff.2025.01325" xr:uid="{90091F37-B8BD-4BFC-A019-906839FABFB8}"/>
+    <hyperlink ref="C128" r:id="rId127" display="https://www.healthaffairs.org/content/forefront/states-exceeding-their-health-care-cost-growth-targets-does-mean" xr:uid="{07B09092-E3BB-4060-80CB-4D88E106A619}"/>
+    <hyperlink ref="C129" r:id="rId128" display="https://www.healthaffairs.org/content/forefront/why-new-drugs-and-ai-chatbots-won-t-cure-health-care-s-cost-disease" xr:uid="{4F073D69-1937-4F8D-8868-0CBA2A6219A7}"/>
+    <hyperlink ref="C130" r:id="rId129" display="https://www.healthaffairs.org/doi/10.1377/hlthaff.2026.00749" xr:uid="{3FAA25BD-2508-45E7-9827-E195A9CE2164}"/>
+    <hyperlink ref="C131" r:id="rId130" display="https://www.healthaffairs.org/content/forefront/cost-effectiveness-thresholds-overvaluing-innovation-undervaluing-health" xr:uid="{EC5E9BE7-5C6E-4049-A64D-C590235C2176}"/>
+    <hyperlink ref="C132" r:id="rId131" display="https://www.healthaffairs.org/content/forefront/levels-growth-and-semantics-role-prices-driving-health-care-spending" xr:uid="{1DD36C96-2124-485D-B38E-FD12539A44C2}"/>
+    <hyperlink ref="C133" r:id="rId132" display="https://www.healthaffairs.org/content/forefront/medicare-s-unrealized-opportunity-using-acos-create-real-competition" xr:uid="{A1AD029D-39C2-4AF6-8D1D-D213C93D7D93}"/>
+    <hyperlink ref="C134" r:id="rId133" display="https://www.healthaffairs.org/content/forefront/us-health-spending-problem-still-prices" xr:uid="{28D17A2C-13E5-42A2-BFB6-0A65FD4FFB24}"/>
+    <hyperlink ref="C4" r:id="rId134" xr:uid="{E1BAF727-8FE2-4017-BD4A-18813BC2FB6F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId136"/>
+    <tablePart r:id="rId135"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>